<commit_message>
Rebuild RM stock workbook with Tapi production entered 30-Oct 05:53 UTC
First build went stale during verification (one back-dated Tapi
production). Adds a check-with-plant note for 4 Lepakshi full coils.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FhJrkS2zi7vtERXC9Qxxvg
</commit_message>
<xml_diff>
--- a/reports/RM-Stock-Plantwise-2026-10-30.xlsx
+++ b/reports/RM-Stock-Plantwise-2026-10-30.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -520,7 +520,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entries to 29-Oct)</t>
+          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entered to 30-Oct 05:53 UTC)</t>
         </is>
       </c>
     </row>
@@ -688,19 +688,19 @@
         <v>162.445</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>256.817</v>
+        <v>232.381</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>419.262</v>
+        <v>394.826</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>11.188</v>
+        <v>11.21</v>
       </c>
     </row>
     <row r="9">
@@ -717,19 +717,19 @@
         <v>973.6799999999999</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>981</v>
+        <v>976</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1219.202</v>
+        <v>1194.766</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>2192.882</v>
+        <v>2168.446</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2365</v>
+        <v>2370</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>171.423</v>
+        <v>171.445</v>
       </c>
     </row>
     <row r="11">
@@ -771,6 +771,20 @@
       <c r="A16" s="9" t="inlineStr">
         <is>
           <t>• Plant = the plant set at Coil Inward and inherited by its baby coils. Deleted rows excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>CHECK WITH PLANT: 4 Lepakshi full coils (LEP-0826-18, LEP-0826-22, LEP-0926-28, LEP-0926-54 = 98.315 MT) have production</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  booked against baby coils that were later deleted from the app — they may already be slit, so Lepakshi full coils may be overstated.</t>
         </is>
       </c>
     </row>
@@ -810,7 +824,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entries to 29-Oct)</t>
+          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entered to 30-Oct 05:53 UTC)</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3474,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entries to 29-Oct)</t>
+          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entered to 30-Oct 05:53 UTC)</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4172,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entries to 29-Oct)</t>
+          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entered to 30-Oct 05:53 UTC)</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5190,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entries to 29-Oct)</t>
+          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entered to 30-Oct 05:53 UTC)</t>
         </is>
       </c>
     </row>
@@ -5547,10 +5561,10 @@
       </c>
       <c r="C23" s="4" t="inlineStr"/>
       <c r="D23" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>26.358</v>
+        <v>1.922</v>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
@@ -6167,10 +6181,10 @@
       <c r="B54" s="13" t="inlineStr"/>
       <c r="C54" s="13" t="inlineStr"/>
       <c r="D54" s="13" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E54" s="14" t="n">
-        <v>256.817</v>
+        <v>232.381</v>
       </c>
       <c r="F54" s="13" t="inlineStr"/>
     </row>
@@ -6184,7 +6198,7 @@
       <c r="C56" s="16" t="inlineStr"/>
       <c r="D56" s="16" t="inlineStr"/>
       <c r="E56" s="17" t="n">
-        <v>419.262</v>
+        <v>394.826</v>
       </c>
       <c r="F56" s="16" t="inlineStr"/>
     </row>
@@ -6227,7 +6241,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entries to 29-Oct)</t>
+          <t>Live data as of 30-Oct-2026 (coil inward / slitting to 30-Oct, production entered to 30-Oct 05:53 UTC)</t>
         </is>
       </c>
     </row>

</xml_diff>